<commit_message>
updated on 25 august
</commit_message>
<xml_diff>
--- a/12625004.xlsx
+++ b/12625004.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/0eb0b81235d0062c/Documents/GitHub/CAP776/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/0eb0b81235d0062c/Desktop/776/CAP776/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="7" documentId="8_{E03027F0-8265-43BF-A0A2-E202A7C3F2C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8CB48B2D-383E-460E-8D18-AB283392070A}"/>
+  <xr:revisionPtr revIDLastSave="19" documentId="8_{E03027F0-8265-43BF-A0A2-E202A7C3F2C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8EA4342B-FFEE-4798-8B09-02956AA72E77}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="500" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="140" uniqueCount="66">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -231,6 +231,9 @@
   <si>
     <t>I am feeling relaxed</t>
   </si>
+  <si>
+    <t>felt bit nervous</t>
+  </si>
 </sst>
 </file>
 
@@ -416,29 +419,17 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="3">
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-        <name val="Arial"/>
-        <charset val="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="2">
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -542,10 +533,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -933,74 +920,74 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="21.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="19" t="s">
+      <c r="A1" s="20" t="s">
         <v>29</v>
       </c>
-      <c r="B1" s="19"/>
-      <c r="C1" s="19"/>
-      <c r="D1" s="19"/>
-      <c r="E1" s="19"/>
-      <c r="F1" s="19"/>
-      <c r="G1" s="19"/>
-      <c r="H1" s="19"/>
-      <c r="I1" s="19"/>
-      <c r="J1" s="19"/>
-      <c r="K1" s="19"/>
-      <c r="L1" s="19"/>
-      <c r="M1" s="19"/>
-      <c r="N1" s="19"/>
+      <c r="B1" s="20"/>
+      <c r="C1" s="20"/>
+      <c r="D1" s="20"/>
+      <c r="E1" s="20"/>
+      <c r="F1" s="20"/>
+      <c r="G1" s="20"/>
+      <c r="H1" s="20"/>
+      <c r="I1" s="20"/>
+      <c r="J1" s="20"/>
+      <c r="K1" s="20"/>
+      <c r="L1" s="20"/>
+      <c r="M1" s="20"/>
+      <c r="N1" s="20"/>
     </row>
     <row r="2" spans="1:14" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="B2" s="20" t="s">
+      <c r="B2" s="21" t="s">
         <v>50</v>
       </c>
-      <c r="C2" s="20"/>
-      <c r="D2" s="20"/>
+      <c r="C2" s="21"/>
+      <c r="D2" s="21"/>
       <c r="E2" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="F2" s="20">
+      <c r="F2" s="21">
         <v>12625004</v>
       </c>
-      <c r="G2" s="20"/>
+      <c r="G2" s="21"/>
     </row>
     <row r="3" spans="1:14" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="B3" s="20" t="s">
+      <c r="B3" s="21" t="s">
         <v>52</v>
       </c>
-      <c r="C3" s="20"/>
-      <c r="D3" s="20"/>
+      <c r="C3" s="21"/>
+      <c r="D3" s="21"/>
       <c r="E3" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="F3" s="20" t="s">
+      <c r="F3" s="21" t="s">
         <v>51</v>
       </c>
-      <c r="G3" s="20"/>
+      <c r="G3" s="21"/>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="A4" s="18" t="s">
+      <c r="A4" s="19" t="s">
         <v>34</v>
       </c>
-      <c r="B4" s="18"/>
-      <c r="C4" s="18"/>
-      <c r="D4" s="18"/>
-      <c r="E4" s="18"/>
-      <c r="F4" s="18"/>
-      <c r="G4" s="18"/>
-      <c r="H4" s="18"/>
-      <c r="I4" s="18"/>
-      <c r="J4" s="18"/>
-      <c r="K4" s="18"/>
-      <c r="L4" s="18"/>
-      <c r="M4" s="18"/>
-      <c r="N4" s="18"/>
+      <c r="B4" s="19"/>
+      <c r="C4" s="19"/>
+      <c r="D4" s="19"/>
+      <c r="E4" s="19"/>
+      <c r="F4" s="19"/>
+      <c r="G4" s="19"/>
+      <c r="H4" s="19"/>
+      <c r="I4" s="19"/>
+      <c r="J4" s="19"/>
+      <c r="K4" s="19"/>
+      <c r="L4" s="19"/>
+      <c r="M4" s="19"/>
+      <c r="N4" s="19"/>
     </row>
     <row r="5" spans="1:14" ht="42" x14ac:dyDescent="0.35">
       <c r="A5" s="7" t="s">
@@ -1333,7 +1320,7 @@
       <c r="M12" s="16" t="s">
         <v>56</v>
       </c>
-      <c r="N12" s="21" t="s">
+      <c r="N12" s="18" t="s">
         <v>64</v>
       </c>
     </row>
@@ -1381,26 +1368,50 @@
       </c>
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="A14" s="13"/>
-      <c r="B14" s="14"/>
-      <c r="C14" s="14"/>
-      <c r="D14" s="14"/>
-      <c r="E14" s="14"/>
-      <c r="F14" s="14"/>
-      <c r="G14" s="14"/>
-      <c r="H14" s="14"/>
-      <c r="I14" s="15" t="str">
+      <c r="A14" s="13">
+        <v>46259</v>
+      </c>
+      <c r="B14" s="14">
+        <v>540</v>
+      </c>
+      <c r="C14" s="14">
+        <v>30</v>
+      </c>
+      <c r="D14" s="14">
+        <v>350</v>
+      </c>
+      <c r="E14" s="14">
+        <v>60</v>
+      </c>
+      <c r="F14" s="14">
+        <v>120</v>
+      </c>
+      <c r="G14" s="14">
+        <v>2</v>
+      </c>
+      <c r="H14" s="14">
+        <v>120</v>
+      </c>
+      <c r="I14" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J14" s="15" t="str">
+        <v>1220</v>
+      </c>
+      <c r="J14" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K14" s="16"/>
-      <c r="L14" s="16"/>
-      <c r="M14" s="16"/>
-      <c r="N14" s="17"/>
+        <v>220</v>
+      </c>
+      <c r="K14" s="16" t="s">
+        <v>59</v>
+      </c>
+      <c r="L14" s="16" t="s">
+        <v>55</v>
+      </c>
+      <c r="M14" s="16" t="s">
+        <v>56</v>
+      </c>
+      <c r="N14" s="17" t="s">
+        <v>65</v>
+      </c>
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A15" s="13"/>
@@ -10089,13 +10100,13 @@
     <mergeCell ref="B3:D3"/>
     <mergeCell ref="F3:G3"/>
   </mergeCells>
-  <conditionalFormatting sqref="J6:J8 J21:J401 J14:J19">
-    <cfRule type="cellIs" dxfId="2" priority="3" operator="lessThan">
+  <conditionalFormatting sqref="J6:J19">
+    <cfRule type="cellIs" dxfId="1" priority="1" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J9:J13">
-    <cfRule type="cellIs" dxfId="0" priority="1" operator="lessThan">
+  <conditionalFormatting sqref="J21:J401">
+    <cfRule type="cellIs" dxfId="0" priority="3" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>